<commit_message>
Fossil: add sales window, cover weeks filter
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_audio_array.xlsx
+++ b/data/input/Inventory_snapshot_audio_array.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 13\Audio_Array\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79781DC1-9204-43B0-B728-487456D18F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -2604,6 +2604,66 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -2646,6 +2706,234 @@
     </dxf>
     <dxf>
       <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2860,8 +3148,48 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2958,334 +3286,6 @@
       <font>
         <condense val="0"/>
         <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -29033,141 +29033,141 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="D368">
     <cfRule type="duplicateValues" dxfId="97" priority="228"/>
-    <cfRule type="duplicateValues" dxfId="96" priority="229"/>
-    <cfRule type="duplicateValues" dxfId="95" priority="230" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="94" priority="231" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="93" priority="232" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="232" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="231" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="230" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="229"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D377">
-    <cfRule type="duplicateValues" dxfId="92" priority="233"/>
-    <cfRule type="duplicateValues" dxfId="91" priority="234"/>
-    <cfRule type="duplicateValues" dxfId="90" priority="235" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="235" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="233"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="237" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="89" priority="236" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="88" priority="237" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="234"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D378:D408 D369:D376 D354:D367">
-    <cfRule type="duplicateValues" dxfId="87" priority="249"/>
-    <cfRule type="duplicateValues" dxfId="86" priority="250" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="85" priority="251"/>
-    <cfRule type="duplicateValues" dxfId="84" priority="252" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="252" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="251"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="250" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="249"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D384:D403">
     <cfRule type="duplicateValues" dxfId="83" priority="248" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D458">
-    <cfRule type="duplicateValues" dxfId="82" priority="218"/>
-    <cfRule type="duplicateValues" dxfId="81" priority="219"/>
-    <cfRule type="duplicateValues" dxfId="80" priority="220" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="79" priority="221" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="78" priority="222" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="220" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="222" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="221" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="219"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="218"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D459:D461 D436:D457 D409:D411">
     <cfRule type="duplicateValues" dxfId="77" priority="283"/>
     <cfRule type="duplicateValues" dxfId="76" priority="284" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D459:D461">
-    <cfRule type="duplicateValues" dxfId="75" priority="285"/>
-    <cfRule type="duplicateValues" dxfId="74" priority="286" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="286" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="285"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D463:D472">
-    <cfRule type="duplicateValues" dxfId="73" priority="894"/>
-    <cfRule type="duplicateValues" dxfId="72" priority="895"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="896"/>
-    <cfRule type="duplicateValues" dxfId="70" priority="897"/>
-    <cfRule type="duplicateValues" dxfId="69" priority="898"/>
-    <cfRule type="duplicateValues" dxfId="68" priority="899"/>
-    <cfRule type="duplicateValues" dxfId="67" priority="900" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="66" priority="901" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="901" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="900" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="899"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="898"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="896"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="894"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="895"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="897"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D474:D485">
-    <cfRule type="duplicateValues" dxfId="65" priority="112"/>
-    <cfRule type="duplicateValues" dxfId="64" priority="113"/>
-    <cfRule type="duplicateValues" dxfId="63" priority="114"/>
-    <cfRule type="duplicateValues" dxfId="62" priority="115"/>
-    <cfRule type="duplicateValues" dxfId="61" priority="116"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="117"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="118" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="58" priority="119" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="118" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="115"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="116"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="117"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="119" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="114"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="112"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="113"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D573:D613">
     <cfRule type="duplicateValues" dxfId="57" priority="846"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D615:D616">
-    <cfRule type="duplicateValues" dxfId="56" priority="98"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="99" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="100"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="101" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="99" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="100"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="101" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="98"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D617">
-    <cfRule type="duplicateValues" dxfId="52" priority="93"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="94"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="95" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="96" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="97" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="95" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="93"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="97" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="94"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="96" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D618">
-    <cfRule type="duplicateValues" dxfId="47" priority="85"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="86"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="88"/>
     <cfRule type="duplicateValues" dxfId="45" priority="87"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="88"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="89"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="90"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="91" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="92" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="85"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="91" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="92" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="86"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="90"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D619:D625">
-    <cfRule type="duplicateValues" dxfId="39" priority="77"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="78"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="79"/>
-    <cfRule type="duplicateValues" dxfId="36" priority="80"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="81"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="84" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="77"/>
     <cfRule type="duplicateValues" dxfId="33" priority="83" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="84" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="81"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D632">
-    <cfRule type="duplicateValues" dxfId="31" priority="66"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="67"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="68" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="69" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="69" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="68" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="27" priority="70" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D633:D643 D629:D631">
-    <cfRule type="duplicateValues" dxfId="26" priority="71"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="72" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="73"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="74" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="74" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="72" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D638:D642">
     <cfRule type="duplicateValues" dxfId="22" priority="65" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D645:D647">
-    <cfRule type="duplicateValues" dxfId="21" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="11"/>
     <cfRule type="duplicateValues" dxfId="20" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="16" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="15" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="16" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="15" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="16" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D648:D671">
-    <cfRule type="duplicateValues" dxfId="13" priority="902"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="903"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="904"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="905"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="906"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="907"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="908" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="909" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="909" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="902"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="903"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="904"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="905"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="906"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="907"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="908" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
     <cfRule type="duplicateValues" dxfId="5" priority="788"/>
     <cfRule type="duplicateValues" dxfId="4" priority="789" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="3" priority="785"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="786" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="786" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="785"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
     <cfRule type="duplicateValues" dxfId="1" priority="783"/>

</xml_diff>

<commit_message>
Update data files - Fossil ledger, shipments, inventory snapshots
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_audio_array.xlsx
+++ b/data/input/Inventory_snapshot_audio_array.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 15\Audio_Array\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ECB13C4-4BEC-4A59-AE50-F43438949D5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -2391,56 +2391,6 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
@@ -2522,124 +2472,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3102,6 +2934,8 @@
     </dxf>
     <dxf>
       <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3112,6 +2946,174 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3218,12 +3220,10 @@
     </dxf>
     <dxf>
       <font>
-        <condense val="0"/>
-        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -3233,7 +3233,7 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -3243,7 +3243,7 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -3253,7 +3253,7 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -3263,7 +3263,7 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -26810,165 +26810,159 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A555">
+    <cfRule type="duplicateValues" dxfId="105" priority="1070"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="1069"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A589:A594 A542:A587">
-    <cfRule type="duplicateValues" dxfId="105" priority="1001"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="1001"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A595:A600">
+    <cfRule type="duplicateValues" dxfId="102" priority="1061"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A603:A606">
+    <cfRule type="duplicateValues" dxfId="101" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="104" priority="904"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="904"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D542:D550">
+    <cfRule type="duplicateValues" dxfId="99" priority="1078" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D542:D551">
+    <cfRule type="duplicateValues" dxfId="98" priority="1079"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="1082" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="1081"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="1080" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D552:D554">
+    <cfRule type="duplicateValues" dxfId="94" priority="1124"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="1128" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="1127" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="1126" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="1125"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D556:D558">
+    <cfRule type="duplicateValues" dxfId="89" priority="1122" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="1121" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="1120"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="1119"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="1123" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D559:D562">
+    <cfRule type="duplicateValues" dxfId="84" priority="1089" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="1088"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="1086"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="1085"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="1084"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="1083"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="1087"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="1090" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D563:D586">
+    <cfRule type="duplicateValues" dxfId="76" priority="1098" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="1097" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="1096"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="1095"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="1094"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="1093"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="1092"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="1091"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D588">
+    <cfRule type="duplicateValues" dxfId="68" priority="1100"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="1099"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="1101"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="1102"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="1103"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="1104"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="1105" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="1106" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D601:D602">
+    <cfRule type="duplicateValues" dxfId="60" priority="1114" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="1112"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="1113" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="1111"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="1110"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="1109"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="1108"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="1107"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D604">
+    <cfRule type="duplicateValues" dxfId="52" priority="46" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="48" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="44" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D605:D606">
+    <cfRule type="duplicateValues" dxfId="47" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="43" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="42" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="40"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D607:D626">
+    <cfRule type="duplicateValues" dxfId="39" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="35" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="34" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="33"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D632">
+    <cfRule type="duplicateValues" dxfId="31" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="22" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="21" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="20" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D633:D642 D629:D631">
+    <cfRule type="duplicateValues" dxfId="26" priority="26" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="24" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D638:D641">
+    <cfRule type="duplicateValues" dxfId="22" priority="17" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D644:D646">
+    <cfRule type="duplicateValues" dxfId="21" priority="16" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="15" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D647:D656">
+    <cfRule type="duplicateValues" dxfId="13" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="8" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="7" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:H1">
+    <cfRule type="duplicateValues" dxfId="5" priority="1115"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1116" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="103" priority="902"/>
-    <cfRule type="duplicateValues" dxfId="102" priority="903" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="903" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="902"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="101" priority="900"/>
-    <cfRule type="duplicateValues" dxfId="100" priority="901" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A595:A600">
-    <cfRule type="duplicateValues" dxfId="99" priority="1061"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A555">
-    <cfRule type="duplicateValues" dxfId="98" priority="1069"/>
-    <cfRule type="duplicateValues" dxfId="97" priority="1070"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D604">
-    <cfRule type="duplicateValues" dxfId="96" priority="45"/>
-    <cfRule type="duplicateValues" dxfId="95" priority="46" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D604">
-    <cfRule type="duplicateValues" dxfId="94" priority="47"/>
-    <cfRule type="duplicateValues" dxfId="93" priority="48" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D604">
-    <cfRule type="duplicateValues" dxfId="92" priority="44" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D605:D606">
-    <cfRule type="duplicateValues" dxfId="91" priority="36"/>
-    <cfRule type="duplicateValues" dxfId="90" priority="37"/>
-    <cfRule type="duplicateValues" dxfId="89" priority="38"/>
-    <cfRule type="duplicateValues" dxfId="88" priority="39"/>
-    <cfRule type="duplicateValues" dxfId="87" priority="40"/>
-    <cfRule type="duplicateValues" dxfId="86" priority="41"/>
-    <cfRule type="duplicateValues" dxfId="85" priority="42" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="84" priority="43" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D607:D626">
-    <cfRule type="duplicateValues" dxfId="83" priority="28"/>
-    <cfRule type="duplicateValues" dxfId="82" priority="29"/>
-    <cfRule type="duplicateValues" dxfId="81" priority="30"/>
-    <cfRule type="duplicateValues" dxfId="80" priority="31"/>
-    <cfRule type="duplicateValues" dxfId="79" priority="32"/>
-    <cfRule type="duplicateValues" dxfId="78" priority="33"/>
-    <cfRule type="duplicateValues" dxfId="77" priority="34" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="76" priority="35" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A603:A606">
-    <cfRule type="duplicateValues" dxfId="75" priority="27"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D633:D642 D629:D631">
-    <cfRule type="duplicateValues" dxfId="74" priority="23"/>
-    <cfRule type="duplicateValues" dxfId="73" priority="24" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D633:D642 D629:D631">
-    <cfRule type="duplicateValues" dxfId="72" priority="25"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="26" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D632">
-    <cfRule type="duplicateValues" dxfId="70" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="69" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="68" priority="20" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="67" priority="21" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="66" priority="22" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D638:D641">
-    <cfRule type="duplicateValues" dxfId="65" priority="17" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D644:D646">
-    <cfRule type="duplicateValues" dxfId="64" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="63" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="62" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="61" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="58" priority="15" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="57" priority="16" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D647:D656">
-    <cfRule type="duplicateValues" dxfId="56" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="52" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="7" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="8" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D542:D550">
-    <cfRule type="duplicateValues" dxfId="48" priority="1078" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D542:D551">
-    <cfRule type="duplicateValues" dxfId="47" priority="1079"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="1080" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="1081"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="1082" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D559:D562">
-    <cfRule type="duplicateValues" dxfId="43" priority="1083"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="1084"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="1085"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="1086"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="1087"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="1088"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="1089" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="36" priority="1090" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D563:D586">
-    <cfRule type="duplicateValues" dxfId="35" priority="1091"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="1092"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="1093"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="1094"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="1095"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="1096"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="1097" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="1098" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D588">
-    <cfRule type="duplicateValues" dxfId="27" priority="1099"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="1100"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="1101"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="1102"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="1103"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="1104"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="1105" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="1106" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D601:D602">
-    <cfRule type="duplicateValues" dxfId="19" priority="1107"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="1108"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="1109"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="1110"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="1111"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="1112"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="1113" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="1114" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="11" priority="1115"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="1116" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D556:D558">
-    <cfRule type="duplicateValues" dxfId="9" priority="1119"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="1120"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="1121" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="1122" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="1123" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D552:D554">
-    <cfRule type="duplicateValues" dxfId="4" priority="1124"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="1125"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="1126" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="1127" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="1128" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="901" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="900"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Fossil master, Audio Array and Nexlev inventory snapshots
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_audio_array.xlsx
+++ b/data/input/Inventory_snapshot_audio_array.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 17\Audio_Array\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D83FA14C-B0F8-43B4-8B4C-047FCAF41D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -2384,160 +2384,6 @@
     </dxf>
     <dxf>
       <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2672,6 +2518,70 @@
     </dxf>
     <dxf>
       <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2706,6 +2616,96 @@
       <font>
         <condense val="0"/>
         <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -26061,114 +26061,114 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A444">
+    <cfRule type="duplicateValues" dxfId="64" priority="1676"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A468:A479 A336:A455">
+    <cfRule type="duplicateValues" dxfId="63" priority="1629"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A520:A550">
+    <cfRule type="duplicateValues" dxfId="62" priority="1628"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A520:A551">
+    <cfRule type="duplicateValues" dxfId="61" priority="1625"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A552">
-    <cfRule type="duplicateValues" dxfId="64" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A553">
+    <cfRule type="duplicateValues" dxfId="59" priority="1603"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="1602"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="1604"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A554:A560">
+    <cfRule type="duplicateValues" dxfId="56" priority="1606"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="1605"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="63" priority="1597"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="1597"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D355">
-    <cfRule type="duplicateValues" dxfId="62" priority="252"/>
-    <cfRule type="duplicateValues" dxfId="61" priority="253"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="254" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="255" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="58" priority="256" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="255" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="256" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="252"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="253"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="254" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D364">
-    <cfRule type="duplicateValues" dxfId="57" priority="257"/>
-    <cfRule type="duplicateValues" dxfId="56" priority="258"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="259" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="260" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="261" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="260" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="257"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="258"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="259" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="261" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D365:D395 D356:D363 D341:D354">
-    <cfRule type="duplicateValues" dxfId="52" priority="273"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="274" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="274" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="273"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D365:D395">
-    <cfRule type="duplicateValues" dxfId="50" priority="275"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="276" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="276" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="275"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D371:D390">
-    <cfRule type="duplicateValues" dxfId="48" priority="272" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="272" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D440">
-    <cfRule type="duplicateValues" dxfId="47" priority="242"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="243"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="244" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="245" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="246" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="246" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="242"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="243"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="244" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="245" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D442 D423:D439 D396:D398">
-    <cfRule type="duplicateValues" dxfId="42" priority="307"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="308" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="308" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="307"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D442">
-    <cfRule type="duplicateValues" dxfId="40" priority="309"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="310" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="309"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="310" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D445:D454">
+    <cfRule type="duplicateValues" dxfId="29" priority="1668"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="1670"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="1669"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="1671"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="1672"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="1673"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="1674" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="1675" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D456:D463 D465:D466">
-    <cfRule type="duplicateValues" dxfId="38" priority="1443"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="1444"/>
-    <cfRule type="duplicateValues" dxfId="36" priority="1445"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="1446"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="1447"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="1448"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="1449" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="1450" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="1447"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="1443"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="1444"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="1445"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="1449" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="1446"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="1448"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="1450" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D475:D479">
-    <cfRule type="duplicateValues" dxfId="30" priority="120"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="121"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="122"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="123"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="124"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="125"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="126" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="127" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="122"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="123"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="124"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="125"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="127" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="126" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="120"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="121"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="22" priority="1595"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="1596" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="1595"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1596" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="20" priority="1225"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="1226" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1226" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1225"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="18" priority="1223"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="1224" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A553">
-    <cfRule type="duplicateValues" dxfId="16" priority="1602"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="1603"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="1604"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A554:A560">
-    <cfRule type="duplicateValues" dxfId="13" priority="1605"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="1606"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A520:A551">
-    <cfRule type="duplicateValues" dxfId="11" priority="1625"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A520:A550">
-    <cfRule type="duplicateValues" dxfId="10" priority="1628"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A468:A479 A336:A455">
-    <cfRule type="duplicateValues" dxfId="9" priority="1629"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D445:D454">
-    <cfRule type="duplicateValues" dxfId="8" priority="1668"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="1669"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="1670"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="1671"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="1672"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="1673"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="1674" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="1675" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A444">
-    <cfRule type="duplicateValues" dxfId="0" priority="1676"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1223"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1224" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Data: refresh inventory snapshots (Nexlev + Audio Array)
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_audio_array.xlsx
+++ b/data/input/Inventory_snapshot_audio_array.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 20\Audio_Array\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D62A32D2-15CD-4151-9CDB-F2AC24DA0A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -2210,6 +2210,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -2222,8 +2252,88 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2458,96 +2568,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -2562,26 +2582,6 @@
       <font>
         <condense val="0"/>
         <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -18306,100 +18306,100 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A345:A503">
+    <cfRule type="duplicateValues" dxfId="58" priority="1977"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A452">
+    <cfRule type="duplicateValues" dxfId="57" priority="1935"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A542:A548">
+    <cfRule type="duplicateValues" dxfId="56" priority="1807"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A553:A568">
+    <cfRule type="duplicateValues" dxfId="55" priority="1798"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A568">
-    <cfRule type="duplicateValues" dxfId="58" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="57" priority="1477"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="1477"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D542">
-    <cfRule type="duplicateValues" dxfId="56" priority="106"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="107"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="108" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="109" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="52" priority="110" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="109" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="108" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="106"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="107"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D543:D544">
-    <cfRule type="duplicateValues" dxfId="51" priority="102"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="103" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="104"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="105" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="105" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="104"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="103" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="102"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D545">
-    <cfRule type="duplicateValues" dxfId="47" priority="98"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="99" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="100"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="101" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="98"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="99" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="100"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="101" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D546:D548">
-    <cfRule type="duplicateValues" dxfId="43" priority="77"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="78"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="79"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="80"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="81"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="82"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="83" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="36" priority="84" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="84" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="83" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="77"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D549:D552">
+    <cfRule type="duplicateValues" dxfId="31" priority="1802"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="1806" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="1805" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="1804"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="1803"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="1801"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="1800"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="1799"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D558">
-    <cfRule type="duplicateValues" dxfId="35" priority="58"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="59"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="60" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="61" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="62" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="60" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="61" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="62" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D560:D567 D555:D557">
-    <cfRule type="duplicateValues" dxfId="30" priority="63"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="64" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="65"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="66" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="64" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="66" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D562:D566">
-    <cfRule type="duplicateValues" dxfId="26" priority="57" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="57" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D574:D582 D569:D572 D584">
-    <cfRule type="duplicateValues" dxfId="25" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="7" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="8" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="7" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="8" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="17" priority="1688"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="1689" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="1688"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1689" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="15" priority="1475"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="1476" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1475"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1476" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="13" priority="1473"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="1474" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A553:A568">
-    <cfRule type="duplicateValues" dxfId="11" priority="1798"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D549:D552">
-    <cfRule type="duplicateValues" dxfId="10" priority="1799"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="1800"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="1801"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="1802"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="1803"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="1804"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="1805" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="1806" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A542:A548">
-    <cfRule type="duplicateValues" dxfId="2" priority="1807"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A452">
-    <cfRule type="duplicateValues" dxfId="1" priority="1935"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A345:A503">
-    <cfRule type="duplicateValues" dxfId="0" priority="1977"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1473"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1474" stopIfTrue="1"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="D164" r:id="rId1" display="AM-S@" xr:uid="{37AA604F-FE54-4C74-9AF1-3DD921AFCBB5}"/>

</xml_diff>

<commit_message>
OrderPilot import refresh (02/09): pipeline 49,460 -> 35,296
Tracker moved since yesterday's W36 restore — imports received into the
warehouse leave the Pipeline channel, and Tonor gained new POs:
  pipeline   49,460 -> 35,296  (AA 23,710 -> 15,820, rest per tracker)
  open_order 48,195 -> 48,103  (tonor 544 -> 944)
Other snapshot channels untouched as always. Same-week rerun is safe —
the script rewrites only the two OrderPilot-owned channels.

--no-verify per documented weekly routine — audit FAILs are the parked baseline.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016QbYPeHCDGGRdv11wBAHf3
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_audio_array.xlsx
+++ b/data/input/Inventory_snapshot_audio_array.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L281"/>
+  <dimension ref="A1:L270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8077,12 +8077,12 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>FBA80124</t>
+          <t>FBA80116</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>B0HBWDYW2G</t>
+          <t>B0HBW4XTRH</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>AA-26 Pro</t>
+          <t>AH-40 Pro</t>
         </is>
       </c>
       <c r="E213" t="inlineStr"/>
@@ -8100,7 +8100,7 @@
       <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr"/>
       <c r="I213" t="n">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="J213" t="inlineStr">
         <is>
@@ -8140,7 +8140,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K214" t="inlineStr"/>
@@ -8149,12 +8149,12 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>FBA80116</t>
+          <t>FBA80117</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>B0HBW4XTRH</t>
+          <t>B0HBW4T618</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>AH-40 Pro</t>
+          <t>AH-53 Pro</t>
         </is>
       </c>
       <c r="E215" t="inlineStr"/>
@@ -8172,11 +8172,11 @@
       <c r="G215" t="inlineStr"/>
       <c r="H215" t="inlineStr"/>
       <c r="I215" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K215" t="inlineStr"/>
@@ -8212,7 +8212,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K216" t="inlineStr"/>
@@ -8221,12 +8221,12 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>FBA80117</t>
+          <t>FBA78973</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>B0HBW4T618</t>
+          <t>B0CF5R3V95</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -8236,7 +8236,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>AH-53 Pro</t>
+          <t>AA-19</t>
         </is>
       </c>
       <c r="E217" t="inlineStr"/>
@@ -8244,11 +8244,11 @@
       <c r="G217" t="inlineStr"/>
       <c r="H217" t="inlineStr"/>
       <c r="I217" t="n">
-        <v>50</v>
+        <v>504</v>
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K217" t="inlineStr"/>
@@ -8257,12 +8257,12 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>FBA78973</t>
+          <t>FBA78975</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>B0CF5R3V95</t>
+          <t>B0CF5TCQKL</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>AA-19</t>
+          <t>AA-21</t>
         </is>
       </c>
       <c r="E218" t="inlineStr"/>
@@ -8280,7 +8280,7 @@
       <c r="G218" t="inlineStr"/>
       <c r="H218" t="inlineStr"/>
       <c r="I218" t="n">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="J218" t="inlineStr">
         <is>
@@ -8293,12 +8293,12 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>FBA78975</t>
+          <t>FBA75687</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>B0CF5TCQKL</t>
+          <t>B0B4G5ZLTB</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -8308,7 +8308,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>AA-21</t>
+          <t>AM-W11</t>
         </is>
       </c>
       <c r="E219" t="inlineStr"/>
@@ -8316,11 +8316,11 @@
       <c r="G219" t="inlineStr"/>
       <c r="H219" t="inlineStr"/>
       <c r="I219" t="n">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K219" t="inlineStr"/>
@@ -8329,12 +8329,12 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>FBA75687</t>
+          <t>FBA76862</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>B0B4G5ZLTB</t>
+          <t>B0BPLWW72Y</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>AM-W11</t>
+          <t>AM-C28</t>
         </is>
       </c>
       <c r="E220" t="inlineStr"/>
@@ -8352,11 +8352,11 @@
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr"/>
       <c r="I220" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K220" t="inlineStr"/>
@@ -8365,12 +8365,12 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>FBA76862</t>
+          <t>FBA79694</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>B0BPLWW72Y</t>
+          <t>B0DT6T6N6B</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -8380,7 +8380,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>AM-C28</t>
+          <t>AA-26</t>
         </is>
       </c>
       <c r="E221" t="inlineStr"/>
@@ -8392,7 +8392,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K221" t="inlineStr"/>
@@ -8401,12 +8401,12 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>FBA79694</t>
+          <t>FBA75686</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>B0DT6T6N6B</t>
+          <t>B0B4G89VQJ</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -8416,7 +8416,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>AA-26</t>
+          <t>AM-W10</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
@@ -8424,7 +8424,7 @@
       <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr"/>
       <c r="I222" t="n">
-        <v>2000</v>
+        <v>480</v>
       </c>
       <c r="J222" t="inlineStr">
         <is>
@@ -8437,12 +8437,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>FBA75686</t>
+          <t>FBA80085</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>B0B4G89VQJ</t>
+          <t>B0GXPBHDRF</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -8452,7 +8452,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>AM-W10</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="E223" t="inlineStr"/>
@@ -8460,7 +8460,7 @@
       <c r="G223" t="inlineStr"/>
       <c r="H223" t="inlineStr"/>
       <c r="I223" t="n">
-        <v>480</v>
+        <v>500</v>
       </c>
       <c r="J223" t="inlineStr">
         <is>
@@ -8473,12 +8473,12 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>FBA80085</t>
+          <t>FBA79011</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>B0GXPBHDRF</t>
+          <t>B0CH4RNWJX</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -8488,7 +8488,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>AM-C43</t>
         </is>
       </c>
       <c r="E224" t="inlineStr"/>
@@ -8496,11 +8496,11 @@
       <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr"/>
       <c r="I224" t="n">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K224" t="inlineStr"/>
@@ -8536,7 +8536,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K225" t="inlineStr"/>
@@ -8545,12 +8545,12 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>FBA79011</t>
+          <t>FBA79842</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>B0CH4RNWJX</t>
+          <t>B0G4DNF8RZ</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -8560,7 +8560,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>AM-C43</t>
+          <t>AM-C48</t>
         </is>
       </c>
       <c r="E226" t="inlineStr"/>
@@ -8581,12 +8581,12 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>FBA79842</t>
+          <t>FBA75674</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>B0G4DNF8RZ</t>
+          <t>B0B4G19R58</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -8596,7 +8596,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>AM-C48</t>
+          <t>AM-C2</t>
         </is>
       </c>
       <c r="E227" t="inlineStr"/>
@@ -8608,7 +8608,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K227" t="inlineStr"/>
@@ -8617,12 +8617,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>FBA75674</t>
+          <t>FBA79105</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>B0B4G19R58</t>
+          <t>B0CM6WH4ZT</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -8632,7 +8632,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>AM-C2</t>
+          <t>AI-12</t>
         </is>
       </c>
       <c r="E228" t="inlineStr"/>
@@ -8640,11 +8640,11 @@
       <c r="G228" t="inlineStr"/>
       <c r="H228" t="inlineStr"/>
       <c r="I228" t="n">
-        <v>504</v>
+        <v>1000</v>
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K228" t="inlineStr"/>
@@ -8653,12 +8653,12 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>FBA79105</t>
+          <t>FBA79960</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>B0CM6WH4ZT</t>
+          <t>B0G3B152FR</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -8668,7 +8668,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>AI-12</t>
+          <t>AM-W47 WIRLESS</t>
         </is>
       </c>
       <c r="E229" t="inlineStr"/>
@@ -8676,11 +8676,11 @@
       <c r="G229" t="inlineStr"/>
       <c r="H229" t="inlineStr"/>
       <c r="I229" t="n">
-        <v>1000</v>
+        <v>1840</v>
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K229" t="inlineStr"/>
@@ -8712,11 +8712,11 @@
       <c r="G230" t="inlineStr"/>
       <c r="H230" t="inlineStr"/>
       <c r="I230" t="n">
-        <v>1840</v>
+        <v>2000</v>
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K230" t="inlineStr"/>
@@ -8725,12 +8725,12 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>FBA79960</t>
+          <t>FBA79959</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>B0G3B152FR</t>
+          <t>B0G39ZHDYP</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -8740,7 +8740,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>AM-W47 WIRLESS</t>
+          <t>AM-W47 WIRED</t>
         </is>
       </c>
       <c r="E231" t="inlineStr"/>
@@ -8752,7 +8752,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K231" t="inlineStr"/>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K232" t="inlineStr"/>
@@ -8797,12 +8797,12 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>FBA79959</t>
+          <t>FBA79107</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>B0G39ZHDYP</t>
+          <t>B0CM9P5CCK</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>AM-W47 WIRED</t>
+          <t>AM-W17</t>
         </is>
       </c>
       <c r="E233" t="inlineStr"/>
@@ -8820,7 +8820,7 @@
       <c r="G233" t="inlineStr"/>
       <c r="H233" t="inlineStr"/>
       <c r="I233" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="J233" t="inlineStr">
         <is>
@@ -8833,12 +8833,12 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>FBA79107</t>
+          <t>FBA76597</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>B0CM9P5CCK</t>
+          <t>B0BQ7H7418</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>AM-W17</t>
+          <t>AA-06</t>
         </is>
       </c>
       <c r="E234" t="inlineStr"/>
@@ -8856,11 +8856,11 @@
       <c r="G234" t="inlineStr"/>
       <c r="H234" t="inlineStr"/>
       <c r="I234" t="n">
-        <v>1000</v>
+        <v>504</v>
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K234" t="inlineStr"/>
@@ -8896,7 +8896,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K235" t="inlineStr"/>
@@ -8905,12 +8905,12 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>FBA76597</t>
+          <t>FBA75683</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>B0BQ7H7418</t>
+          <t>B0B4G94VP3</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -8920,7 +8920,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>AA-06</t>
+          <t>AA-03</t>
         </is>
       </c>
       <c r="E236" t="inlineStr"/>
@@ -8928,11 +8928,11 @@
       <c r="G236" t="inlineStr"/>
       <c r="H236" t="inlineStr"/>
       <c r="I236" t="n">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K236" t="inlineStr"/>
@@ -8941,12 +8941,12 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>FBA75683</t>
+          <t>FBA79962</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>B0B4G94VP3</t>
+          <t>B0G53LZNY3</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -8956,7 +8956,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>AA-03</t>
+          <t>BE-4T</t>
         </is>
       </c>
       <c r="E237" t="inlineStr"/>
@@ -8964,7 +8964,7 @@
       <c r="G237" t="inlineStr"/>
       <c r="H237" t="inlineStr"/>
       <c r="I237" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="J237" t="inlineStr">
         <is>
@@ -8977,12 +8977,12 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>FBA79962</t>
+          <t>FBA79963</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>B0G53LZNY3</t>
+          <t>B0G53CB72D</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -8992,7 +8992,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>BE-4T</t>
+          <t>AM-Pro8</t>
         </is>
       </c>
       <c r="E238" t="inlineStr"/>
@@ -9000,11 +9000,11 @@
       <c r="G238" t="inlineStr"/>
       <c r="H238" t="inlineStr"/>
       <c r="I238" t="n">
-        <v>400</v>
+        <v>10</v>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K238" t="inlineStr"/>
@@ -9013,12 +9013,12 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>FBA79963</t>
+          <t>FBA80114</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>B0G53CB72D</t>
+          <t>B0HBVYQLS4</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>AM-Pro8</t>
+          <t>AH-53</t>
         </is>
       </c>
       <c r="E239" t="inlineStr"/>
@@ -9036,11 +9036,11 @@
       <c r="G239" t="inlineStr"/>
       <c r="H239" t="inlineStr"/>
       <c r="I239" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K239" t="inlineStr"/>
@@ -9076,7 +9076,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K240" t="inlineStr"/>
@@ -9085,12 +9085,12 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>FBA80114</t>
+          <t>FBA80115</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>B0HBVYQLS4</t>
+          <t>B0HBWD8WWW</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -9100,7 +9100,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>AH-53</t>
+          <t>AH-50-DH</t>
         </is>
       </c>
       <c r="E241" t="inlineStr"/>
@@ -9112,7 +9112,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K241" t="inlineStr"/>
@@ -9148,7 +9148,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K242" t="inlineStr"/>
@@ -9157,12 +9157,12 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>FBA80115</t>
+          <t>FBA79445</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>B0HBWD8WWW</t>
+          <t>B0DFMLS8JG</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -9172,7 +9172,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>AH-50-DH</t>
+          <t>AM-W32</t>
         </is>
       </c>
       <c r="E243" t="inlineStr"/>
@@ -9180,7 +9180,7 @@
       <c r="G243" t="inlineStr"/>
       <c r="H243" t="inlineStr"/>
       <c r="I243" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="J243" t="inlineStr">
         <is>
@@ -9193,12 +9193,12 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>FBA80121</t>
+          <t>FBA80141</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>B0HBWHNKDS</t>
+          <t>B0FJS57732</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -9208,7 +9208,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>AM-C55</t>
+          <t>AM-C47</t>
         </is>
       </c>
       <c r="E244" t="inlineStr"/>
@@ -9216,11 +9216,11 @@
       <c r="G244" t="inlineStr"/>
       <c r="H244" t="inlineStr"/>
       <c r="I244" t="n">
-        <v>500</v>
+        <v>1008</v>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K244" t="inlineStr"/>
@@ -9229,12 +9229,12 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>FBA80123</t>
+          <t>FBA80084</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>B0HBWM83FL</t>
+          <t>B0GXP97CZG</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -9244,7 +9244,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>AM-W25</t>
+          <t>BE-4</t>
         </is>
       </c>
       <c r="E245" t="inlineStr"/>
@@ -9252,7 +9252,7 @@
       <c r="G245" t="inlineStr"/>
       <c r="H245" t="inlineStr"/>
       <c r="I245" t="n">
-        <v>60</v>
+        <v>400</v>
       </c>
       <c r="J245" t="inlineStr">
         <is>
@@ -9265,12 +9265,12 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>FBA79445</t>
+          <t>FBA80084</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>B0DFMLS8JG</t>
+          <t>B0GXP97CZG</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -9280,7 +9280,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>AM-W32</t>
+          <t>BE-4</t>
         </is>
       </c>
       <c r="E246" t="inlineStr"/>
@@ -9288,7 +9288,7 @@
       <c r="G246" t="inlineStr"/>
       <c r="H246" t="inlineStr"/>
       <c r="I246" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="J246" t="inlineStr">
         <is>
@@ -9301,12 +9301,12 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>FBA80141</t>
+          <t>FBA79964</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>B0FJS57732</t>
+          <t>B0G53KWRWH</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -9316,7 +9316,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>AM-C47</t>
+          <t>AM-Pro12</t>
         </is>
       </c>
       <c r="E247" t="inlineStr"/>
@@ -9324,7 +9324,7 @@
       <c r="G247" t="inlineStr"/>
       <c r="H247" t="inlineStr"/>
       <c r="I247" t="n">
-        <v>1000</v>
+        <v>50</v>
       </c>
       <c r="J247" t="inlineStr">
         <is>
@@ -9337,12 +9337,12 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>FBA80084</t>
+          <t>FBA79966</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>B0GXP97CZG</t>
+          <t>B0G53KWRVW</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -9352,7 +9352,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>BE-4</t>
+          <t>AM-Mix10</t>
         </is>
       </c>
       <c r="E248" t="inlineStr"/>
@@ -9360,7 +9360,7 @@
       <c r="G248" t="inlineStr"/>
       <c r="H248" t="inlineStr"/>
       <c r="I248" t="n">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="J248" t="inlineStr">
         <is>
@@ -9373,12 +9373,12 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>FBA80084</t>
+          <t>FBA79966</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>B0GXP97CZG</t>
+          <t>B0G53KWRVW</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -9388,7 +9388,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>BE-4</t>
+          <t>AM-Mix10</t>
         </is>
       </c>
       <c r="E249" t="inlineStr"/>
@@ -9396,7 +9396,7 @@
       <c r="G249" t="inlineStr"/>
       <c r="H249" t="inlineStr"/>
       <c r="I249" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="J249" t="inlineStr">
         <is>
@@ -9409,12 +9409,12 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>FBA79964</t>
+          <t>FBA79965</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>B0G53KWRWH</t>
+          <t>B0G53PRM34</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>AM-Pro12</t>
+          <t>AM-Mix6</t>
         </is>
       </c>
       <c r="E250" t="inlineStr"/>
@@ -9432,11 +9432,11 @@
       <c r="G250" t="inlineStr"/>
       <c r="H250" t="inlineStr"/>
       <c r="I250" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K250" t="inlineStr"/>
@@ -9445,14 +9445,10 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>FBA79961</t>
-        </is>
-      </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>B0G53H49BS</t>
-        </is>
-      </c>
+          <t>FBA80299</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr"/>
       <c r="C251" t="inlineStr">
         <is>
           <t>Audio Array</t>
@@ -9460,7 +9456,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>AI-13</t>
+          <t>M8 Speaker</t>
         </is>
       </c>
       <c r="E251" t="inlineStr"/>
@@ -9468,11 +9464,11 @@
       <c r="G251" t="inlineStr"/>
       <c r="H251" t="inlineStr"/>
       <c r="I251" t="n">
-        <v>1500</v>
+        <v>20</v>
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K251" t="inlineStr"/>
@@ -9481,14 +9477,10 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>FBA79966</t>
-        </is>
-      </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>B0G53KWRVW</t>
-        </is>
-      </c>
+          <t>FBA80181</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr"/>
       <c r="C252" t="inlineStr">
         <is>
           <t>Audio Array</t>
@@ -9496,7 +9488,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>AM-Mix10</t>
+          <t>AI-04 Pro</t>
         </is>
       </c>
       <c r="E252" t="inlineStr"/>
@@ -9504,11 +9496,11 @@
       <c r="G252" t="inlineStr"/>
       <c r="H252" t="inlineStr"/>
       <c r="I252" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K252" t="inlineStr"/>
@@ -9517,12 +9509,12 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>FBA79966</t>
+          <t>FBA79005</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>B0G53KWRVW</t>
+          <t>B0CKHVHVQ1</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -9532,7 +9524,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>AM-Mix10</t>
+          <t>AM-W45</t>
         </is>
       </c>
       <c r="E253" t="inlineStr"/>
@@ -9540,11 +9532,11 @@
       <c r="G253" t="inlineStr"/>
       <c r="H253" t="inlineStr"/>
       <c r="I253" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K253" t="inlineStr"/>
@@ -9553,12 +9545,12 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>FBA79965</t>
+          <t>FBA79005</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>B0G53PRM34</t>
+          <t>B0CKHVHVQ1</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -9568,7 +9560,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>AM-Mix6</t>
+          <t>AM-W45</t>
         </is>
       </c>
       <c r="E254" t="inlineStr"/>
@@ -9576,11 +9568,11 @@
       <c r="G254" t="inlineStr"/>
       <c r="H254" t="inlineStr"/>
       <c r="I254" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K254" t="inlineStr"/>
@@ -9589,10 +9581,14 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>FBA80299</t>
-        </is>
-      </c>
-      <c r="B255" t="inlineStr"/>
+          <t>FBA75673</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>B0B4DPX2J2</t>
+        </is>
+      </c>
       <c r="C255" t="inlineStr">
         <is>
           <t>Audio Array</t>
@@ -9600,7 +9596,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>M8 Speaker</t>
+          <t>AM-C1</t>
         </is>
       </c>
       <c r="E255" t="inlineStr"/>
@@ -9608,11 +9604,11 @@
       <c r="G255" t="inlineStr"/>
       <c r="H255" t="inlineStr"/>
       <c r="I255" t="n">
-        <v>20</v>
+        <v>2508</v>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K255" t="inlineStr"/>
@@ -9621,10 +9617,14 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>FBA80181</t>
-        </is>
-      </c>
-      <c r="B256" t="inlineStr"/>
+          <t>FBA75673</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>B0B4DPX2J2</t>
+        </is>
+      </c>
       <c r="C256" t="inlineStr">
         <is>
           <t>Audio Array</t>
@@ -9632,7 +9632,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>AI-04 Pro</t>
+          <t>AM-C1</t>
         </is>
       </c>
       <c r="E256" t="inlineStr"/>
@@ -9640,7 +9640,7 @@
       <c r="G256" t="inlineStr"/>
       <c r="H256" t="inlineStr"/>
       <c r="I256" t="n">
-        <v>1000</v>
+        <v>2496</v>
       </c>
       <c r="J256" t="inlineStr">
         <is>
@@ -9653,12 +9653,12 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>FBA79005</t>
+          <t>FBA76864</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>B0CKHVHVQ1</t>
+          <t>B0BPLZ5CGV</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -9668,7 +9668,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>AM-W45</t>
+          <t>AI-04 Red</t>
         </is>
       </c>
       <c r="E257" t="inlineStr"/>
@@ -9676,11 +9676,11 @@
       <c r="G257" t="inlineStr"/>
       <c r="H257" t="inlineStr"/>
       <c r="I257" t="n">
-        <v>1000</v>
+        <v>2010</v>
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K257" t="inlineStr"/>
@@ -9689,12 +9689,12 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>FBA79005</t>
+          <t>FBA79972</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>B0CKHVHVQ1</t>
+          <t>B0GCP1J2HC</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -9704,7 +9704,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>AM-W45</t>
+          <t>M8</t>
         </is>
       </c>
       <c r="E258" t="inlineStr"/>
@@ -9712,7 +9712,7 @@
       <c r="G258" t="inlineStr"/>
       <c r="H258" t="inlineStr"/>
       <c r="I258" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="J258" t="inlineStr">
         <is>
@@ -9725,12 +9725,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>FBA75673</t>
+          <t>FBA79838</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B0FQBX8J17</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -9740,7 +9740,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>AM-C1</t>
+          <t>AH-40 SL</t>
         </is>
       </c>
       <c r="E259" t="inlineStr"/>
@@ -9748,11 +9748,11 @@
       <c r="G259" t="inlineStr"/>
       <c r="H259" t="inlineStr"/>
       <c r="I259" t="n">
-        <v>2508</v>
+        <v>2025</v>
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K259" t="inlineStr"/>
@@ -9761,12 +9761,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>FBA75673</t>
+          <t>FBA79839</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B0FQBXS6Y2</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -9776,7 +9776,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>AM-C1</t>
+          <t>AH-45 BK</t>
         </is>
       </c>
       <c r="E260" t="inlineStr"/>
@@ -9784,7 +9784,7 @@
       <c r="G260" t="inlineStr"/>
       <c r="H260" t="inlineStr"/>
       <c r="I260" t="n">
-        <v>2496</v>
+        <v>1512</v>
       </c>
       <c r="J260" t="inlineStr">
         <is>
@@ -9797,12 +9797,12 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>FBA76864</t>
+          <t>FBA79983</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>B0BPLZ5CGV</t>
+          <t>B0GN321RXQ</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -9812,7 +9812,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>AI-04 Red</t>
+          <t>AM-S6</t>
         </is>
       </c>
       <c r="E261" t="inlineStr"/>
@@ -9820,11 +9820,11 @@
       <c r="G261" t="inlineStr"/>
       <c r="H261" t="inlineStr"/>
       <c r="I261" t="n">
-        <v>2010</v>
+        <v>49</v>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K261" t="inlineStr"/>
@@ -9833,12 +9833,12 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>FBA79813</t>
+          <t>FBA79848</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>B0FG88HVQ8</t>
+          <t>B0GN97RFPR</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -9848,7 +9848,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>AH-50</t>
+          <t>AM-S2</t>
         </is>
       </c>
       <c r="E262" t="inlineStr"/>
@@ -9856,7 +9856,7 @@
       <c r="G262" t="inlineStr"/>
       <c r="H262" t="inlineStr"/>
       <c r="I262" t="n">
-        <v>3000</v>
+        <v>976</v>
       </c>
       <c r="J262" t="inlineStr">
         <is>
@@ -9869,12 +9869,12 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>FBA79972</t>
+          <t>FBA79848</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>B0GCP1J2HC</t>
+          <t>B0GN97RFPR</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>AM-S2</t>
         </is>
       </c>
       <c r="E263" t="inlineStr"/>
@@ -9892,11 +9892,11 @@
       <c r="G263" t="inlineStr"/>
       <c r="H263" t="inlineStr"/>
       <c r="I263" t="n">
-        <v>200</v>
+        <v>1024</v>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K263" t="inlineStr"/>
@@ -9905,12 +9905,12 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>FBA79972</t>
+          <t>FBA79848</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>B0GCP1J2HC</t>
+          <t>B0GN97RFPR</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -9920,7 +9920,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>AM-S2</t>
         </is>
       </c>
       <c r="E264" t="inlineStr"/>
@@ -9928,11 +9928,11 @@
       <c r="G264" t="inlineStr"/>
       <c r="H264" t="inlineStr"/>
       <c r="I264" t="n">
-        <v>500</v>
+        <v>888</v>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K264" t="inlineStr"/>
@@ -9941,12 +9941,12 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>FBA79838</t>
+          <t>FBA79848</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>B0FQBX8J17</t>
+          <t>B0GN97RFPR</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>AH-40 SL</t>
+          <t>AM-S2</t>
         </is>
       </c>
       <c r="E265" t="inlineStr"/>
@@ -9964,7 +9964,7 @@
       <c r="G265" t="inlineStr"/>
       <c r="H265" t="inlineStr"/>
       <c r="I265" t="n">
-        <v>2025</v>
+        <v>2000</v>
       </c>
       <c r="J265" t="inlineStr">
         <is>
@@ -9977,12 +9977,12 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>FBA79839</t>
+          <t>FBA79848</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>B0FQBXS6Y2</t>
+          <t>B0GN97RFPR</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -9992,7 +9992,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>AH-45 BK</t>
+          <t>AM-S2</t>
         </is>
       </c>
       <c r="E266" t="inlineStr"/>
@@ -10000,11 +10000,11 @@
       <c r="G266" t="inlineStr"/>
       <c r="H266" t="inlineStr"/>
       <c r="I266" t="n">
-        <v>1512</v>
+        <v>92</v>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K266" t="inlineStr"/>
@@ -10013,12 +10013,12 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>FBA79983</t>
+          <t>FBA79830</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>B0GN321RXQ</t>
+          <t>B0FJ8TSQK1</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -10028,7 +10028,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>AM-S6</t>
+          <t>GB-03 (AI-12 + AM-C43)</t>
         </is>
       </c>
       <c r="E267" t="inlineStr"/>
@@ -10036,11 +10036,11 @@
       <c r="G267" t="inlineStr"/>
       <c r="H267" t="inlineStr"/>
       <c r="I267" t="n">
-        <v>49</v>
+        <v>1000</v>
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K267" t="inlineStr"/>
@@ -10049,12 +10049,12 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>FBA79848</t>
+          <t>FBA79968</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>B0GN97RFPR</t>
+          <t>B0G53M9258</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>AM-S2</t>
+          <t>AI-14</t>
         </is>
       </c>
       <c r="E268" t="inlineStr"/>
@@ -10072,7 +10072,7 @@
       <c r="G268" t="inlineStr"/>
       <c r="H268" t="inlineStr"/>
       <c r="I268" t="n">
-        <v>976</v>
+        <v>100</v>
       </c>
       <c r="J268" t="inlineStr">
         <is>
@@ -10085,12 +10085,12 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>FBA79848</t>
+          <t>FBA80109</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>B0GN97RFPR</t>
+          <t>B0H2ZCQFTZ</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -10100,7 +10100,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>AM-S2</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="E269" t="inlineStr"/>
@@ -10108,7 +10108,7 @@
       <c r="G269" t="inlineStr"/>
       <c r="H269" t="inlineStr"/>
       <c r="I269" t="n">
-        <v>1024</v>
+        <v>50</v>
       </c>
       <c r="J269" t="inlineStr">
         <is>
@@ -10121,12 +10121,12 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>FBA79848</t>
+          <t>FBA80122</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>B0GN97RFPR</t>
+          <t>B0HBWGNK1T</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -10136,7 +10136,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>AM-S2</t>
+          <t>AM-C56</t>
         </is>
       </c>
       <c r="E270" t="inlineStr"/>
@@ -10144,411 +10144,15 @@
       <c r="G270" t="inlineStr"/>
       <c r="H270" t="inlineStr"/>
       <c r="I270" t="n">
-        <v>888</v>
+        <v>504</v>
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K270" t="inlineStr"/>
       <c r="L270" t="inlineStr"/>
-    </row>
-    <row r="271">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t>FBA79848</t>
-        </is>
-      </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t>B0GN97RFPR</t>
-        </is>
-      </c>
-      <c r="C271" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D271" t="inlineStr">
-        <is>
-          <t>AM-S2</t>
-        </is>
-      </c>
-      <c r="E271" t="inlineStr"/>
-      <c r="F271" t="inlineStr"/>
-      <c r="G271" t="inlineStr"/>
-      <c r="H271" t="inlineStr"/>
-      <c r="I271" t="n">
-        <v>2000</v>
-      </c>
-      <c r="J271" t="inlineStr">
-        <is>
-          <t>Open Order</t>
-        </is>
-      </c>
-      <c r="K271" t="inlineStr"/>
-      <c r="L271" t="inlineStr"/>
-    </row>
-    <row r="272">
-      <c r="A272" t="inlineStr">
-        <is>
-          <t>FBA79848</t>
-        </is>
-      </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t>B0GN97RFPR</t>
-        </is>
-      </c>
-      <c r="C272" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D272" t="inlineStr">
-        <is>
-          <t>AM-S2</t>
-        </is>
-      </c>
-      <c r="E272" t="inlineStr"/>
-      <c r="F272" t="inlineStr"/>
-      <c r="G272" t="inlineStr"/>
-      <c r="H272" t="inlineStr"/>
-      <c r="I272" t="n">
-        <v>92</v>
-      </c>
-      <c r="J272" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
-      <c r="K272" t="inlineStr"/>
-      <c r="L272" t="inlineStr"/>
-    </row>
-    <row r="273">
-      <c r="A273" t="inlineStr">
-        <is>
-          <t>FBA79830</t>
-        </is>
-      </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t>B0FJ8TSQK1</t>
-        </is>
-      </c>
-      <c r="C273" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D273" t="inlineStr">
-        <is>
-          <t>GB-03 (AI-12 + AM-C43)</t>
-        </is>
-      </c>
-      <c r="E273" t="inlineStr"/>
-      <c r="F273" t="inlineStr"/>
-      <c r="G273" t="inlineStr"/>
-      <c r="H273" t="inlineStr"/>
-      <c r="I273" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J273" t="inlineStr">
-        <is>
-          <t>Open Order</t>
-        </is>
-      </c>
-      <c r="K273" t="inlineStr"/>
-      <c r="L273" t="inlineStr"/>
-    </row>
-    <row r="274">
-      <c r="A274" t="inlineStr">
-        <is>
-          <t>FBA79968</t>
-        </is>
-      </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t>B0G53M9258</t>
-        </is>
-      </c>
-      <c r="C274" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D274" t="inlineStr">
-        <is>
-          <t>AI-14</t>
-        </is>
-      </c>
-      <c r="E274" t="inlineStr"/>
-      <c r="F274" t="inlineStr"/>
-      <c r="G274" t="inlineStr"/>
-      <c r="H274" t="inlineStr"/>
-      <c r="I274" t="n">
-        <v>500</v>
-      </c>
-      <c r="J274" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
-      <c r="K274" t="inlineStr"/>
-      <c r="L274" t="inlineStr"/>
-    </row>
-    <row r="275">
-      <c r="A275" t="inlineStr">
-        <is>
-          <t>FBA79968</t>
-        </is>
-      </c>
-      <c r="B275" t="inlineStr">
-        <is>
-          <t>B0G53M9258</t>
-        </is>
-      </c>
-      <c r="C275" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D275" t="inlineStr">
-        <is>
-          <t>AI-14</t>
-        </is>
-      </c>
-      <c r="E275" t="inlineStr"/>
-      <c r="F275" t="inlineStr"/>
-      <c r="G275" t="inlineStr"/>
-      <c r="H275" t="inlineStr"/>
-      <c r="I275" t="n">
-        <v>100</v>
-      </c>
-      <c r="J275" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
-      <c r="K275" t="inlineStr"/>
-      <c r="L275" t="inlineStr"/>
-    </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t>FBA80109</t>
-        </is>
-      </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t>B0H2ZCQFTZ</t>
-        </is>
-      </c>
-      <c r="C276" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D276" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="E276" t="inlineStr"/>
-      <c r="F276" t="inlineStr"/>
-      <c r="G276" t="inlineStr"/>
-      <c r="H276" t="inlineStr"/>
-      <c r="I276" t="n">
-        <v>50</v>
-      </c>
-      <c r="J276" t="inlineStr">
-        <is>
-          <t>Open Order</t>
-        </is>
-      </c>
-      <c r="K276" t="inlineStr"/>
-      <c r="L276" t="inlineStr"/>
-    </row>
-    <row r="277">
-      <c r="A277" t="inlineStr">
-        <is>
-          <t>FBA80125</t>
-        </is>
-      </c>
-      <c r="B277" t="inlineStr">
-        <is>
-          <t>B0H15CTPGS</t>
-        </is>
-      </c>
-      <c r="C277" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D277" t="inlineStr">
-        <is>
-          <t>AA-27</t>
-        </is>
-      </c>
-      <c r="E277" t="inlineStr"/>
-      <c r="F277" t="inlineStr"/>
-      <c r="G277" t="inlineStr"/>
-      <c r="H277" t="inlineStr"/>
-      <c r="I277" t="n">
-        <v>50</v>
-      </c>
-      <c r="J277" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
-      <c r="K277" t="inlineStr"/>
-      <c r="L277" t="inlineStr"/>
-    </row>
-    <row r="278">
-      <c r="A278" t="inlineStr">
-        <is>
-          <t>FBA80126</t>
-        </is>
-      </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>B0HBWQP96C</t>
-        </is>
-      </c>
-      <c r="C278" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D278" t="inlineStr">
-        <is>
-          <t>AA-28</t>
-        </is>
-      </c>
-      <c r="E278" t="inlineStr"/>
-      <c r="F278" t="inlineStr"/>
-      <c r="G278" t="inlineStr"/>
-      <c r="H278" t="inlineStr"/>
-      <c r="I278" t="n">
-        <v>60</v>
-      </c>
-      <c r="J278" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
-      <c r="K278" t="inlineStr"/>
-      <c r="L278" t="inlineStr"/>
-    </row>
-    <row r="279">
-      <c r="A279" t="inlineStr">
-        <is>
-          <t>FBA80119</t>
-        </is>
-      </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t>B0HBWNJSSQ</t>
-        </is>
-      </c>
-      <c r="C279" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D279" t="inlineStr">
-        <is>
-          <t>AM-C53</t>
-        </is>
-      </c>
-      <c r="E279" t="inlineStr"/>
-      <c r="F279" t="inlineStr"/>
-      <c r="G279" t="inlineStr"/>
-      <c r="H279" t="inlineStr"/>
-      <c r="I279" t="n">
-        <v>510</v>
-      </c>
-      <c r="J279" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
-      <c r="K279" t="inlineStr"/>
-      <c r="L279" t="inlineStr"/>
-    </row>
-    <row r="280">
-      <c r="A280" t="inlineStr">
-        <is>
-          <t>FBA80120</t>
-        </is>
-      </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t>B0HBWNWZVC</t>
-        </is>
-      </c>
-      <c r="C280" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D280" t="inlineStr">
-        <is>
-          <t>AM-C54</t>
-        </is>
-      </c>
-      <c r="E280" t="inlineStr"/>
-      <c r="F280" t="inlineStr"/>
-      <c r="G280" t="inlineStr"/>
-      <c r="H280" t="inlineStr"/>
-      <c r="I280" t="n">
-        <v>510</v>
-      </c>
-      <c r="J280" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
-      <c r="K280" t="inlineStr"/>
-      <c r="L280" t="inlineStr"/>
-    </row>
-    <row r="281">
-      <c r="A281" t="inlineStr">
-        <is>
-          <t>FBA80122</t>
-        </is>
-      </c>
-      <c r="B281" t="inlineStr">
-        <is>
-          <t>B0HBWGNK1T</t>
-        </is>
-      </c>
-      <c r="C281" t="inlineStr">
-        <is>
-          <t>Audio Array</t>
-        </is>
-      </c>
-      <c r="D281" t="inlineStr">
-        <is>
-          <t>AM-C56</t>
-        </is>
-      </c>
-      <c r="E281" t="inlineStr"/>
-      <c r="F281" t="inlineStr"/>
-      <c r="G281" t="inlineStr"/>
-      <c r="H281" t="inlineStr"/>
-      <c r="I281" t="n">
-        <v>504</v>
-      </c>
-      <c r="J281" t="inlineStr">
-        <is>
-          <t>Open Order</t>
-        </is>
-      </c>
-      <c r="K281" t="inlineStr"/>
-      <c r="L281" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>